<commit_message>
docs: add Lee et al. 2026 to multi-judge lit review
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/phase_7.3/Paper Dictionary.xlsx
+++ b/literature-review/phase_7.3/Paper Dictionary.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1292,6 +1292,43 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Judging Against the Reference: Uncovering Knowledge-Driven Failures in LLM-Judges on QA Evaluation</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2601.07506v1</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Identifies a critical failure mode in reference-based LLM QA evaluation: when the provided reference text conflicts with the judge model's parametric (training) knowledge, the judge systematically favors its own prior over the reference, producing unreliable scores. Constructs a benchmark of knowledge-conflicting QA pairs to study this phenomenon and shows it substantially degrades evaluation fidelity across multiple judge models.</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Directly relevant to criteria-grounded factual verification against source text (Phase 7.3 Q4). 2026 paper. Identifies a concrete, testable failure mode — not a vague bias concern. Provides a clear mitigation direction: cross-family judges are less likely to share the same parametric knowledge bias.</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Does not specifically test multi-judge setups as the mitigation. Focuses on QA evaluation fidelity rather than benchmark curation (filtering) tasks. Does not study binary PASS/FAIL rubrics — uses continuous scoring.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>For LectureBench Q4: lecture content (especially cutting-edge ML topics from MIT/Stanford/NYU) may conflict with Claude's parametric knowledge. Lee et al. (2026) argues this is a real failure mode for reference-based judging. The cross-family optional reviewer (GPT-4o) in D1 gains additional justification specifically for Q4 in lectures covering recent or specialized content. This strengthens the case for the optional Kappa reliability check (D8b): if Kappa &lt; 0.7, the disagreements are likely driven by knowledge conflicts, not random noise.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
docs: update lit review Q1-Q6 with peer-reviewed citations
- Add Baysan et al. (Frontiers 2025) and DeCE/Yu et al. (EMNLP 2025)
- Correct Ho et al. arXiv ID; flag as preprint-only
- Remove EduVidQA from Q1 support (hybrid, not LLM-only)
- Add chunk-as-ground-truth argument for LLM-only curation
- Update Q5 with actual run results (398/900 accepted, 56% rejection)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/phase_7.3/Paper Dictionary.xlsx
+++ b/literature-review/phase_7.3/Paper Dictionary.xlsx
@@ -489,11 +489,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
@@ -1329,6 +1329,80 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>LLM-as-a-Judge: Automated Evaluation of Search Query Parsing Using Large Language Models</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.frontiersin.org/journals/big-data/articles/10.3389/fdata.2025.1611389/full</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Proposes an LLM-as-judge framework for structured Pass/Fail evaluation of search query parsing outputs, achieving ~90% agreement with human judgments. Introduces contextual prompt routing to reduce hallucinations. Validated on small- and large-scale datasets in a real-world structured output evaluation setting.</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Peer-reviewed, published in Frontiers in Big Data (2025). Directly validates LLM-based structured Pass/Fail evaluation reliability (~90% human agreement), supporting single-judge structured criteria evaluation for Q1. Closest published analogue to Phase 7.3's binary accept/reject rubric.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Evaluates structured output parsing (JSON), not QA pair correctness. Does not study same-model review or knowledge-conflict failure modes. Domain differs from lecture video QA.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Supports Q1 decision: LLM single-judge is reliable for structured Pass/Fail tasks. Peer-reviewed alternative to the unreviewed Ho et al. (2025) preprint for structured evaluation reliability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Beyond Pointwise Scores: Decomposed Criteria-Based Evaluation of LLM Responses</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>https://aclanthology.org/2025.emnlp-industry.136/</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Introduces DeCE, a decomposed LLM evaluation framework separating precision and recall via instance-specific criteria automatically extracted from gold answers. Applied to legal QA with multi-jurisdictional reasoning and citation grounding, achieving r=0.78 with expert judgments vs r=0.35 for pointwise LLM scoring and r=0.12 for traditional metrics.</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Published at EMNLP 2025 Industry Track (peer-reviewed). Directly validates the G-Eval form-filling / decomposed criteria approach used in Phase 7.3's rubric. Shows decomposed criteria evaluation substantially outperforms pointwise scoring in expert domains (legal QA), which is analogous to structured academic lecture QA.</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Focuses on legal QA, not video lecture QA. Criteria are automatically extracted from gold answers rather than predefined; Phase 7.3 uses fixed predefined criteria. Evaluates answer quality, not benchmark curation filtering.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Supports Q2 decision: decomposed criteria-based evaluation (our G-Eval rubric with Criterion 1/2/3) achieves higher human correlation than holistic pointwise scoring. Peer-reviewed EMNLP 2025 publication strengthens rubric design justification.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
docs: add Venue/Peer-Reviewed column to phase 7.3 Paper Dictionary
Green (✓) for peer-reviewed venues, red (✗) for arXiv preprints.
8 peer-reviewed, 13 preprints, 2 workshop papers across 23 papers.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/phase_7.3/Paper Dictionary.xlsx
+++ b/literature-review/phase_7.3/Paper Dictionary.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +35,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +63,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
         <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -108,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -124,6 +138,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -499,6 +522,7 @@
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -513,6 +537,11 @@
       <c r="E1" s="5" t="n"/>
       <c r="F1" s="5" t="n"/>
       <c r="G1" s="6" t="n"/>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>LLM-as-Judge for QA Benchmark Validation (LectureBench Phase 7.3)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
@@ -551,6 +580,11 @@
           <t>How Current Paper Resolves Gaps</t>
         </is>
       </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Venue / Peer-Reviewed?</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -588,6 +622,11 @@
           <t>LectureBench uses structured checklist prompting (not open-ended) which mitigates self-enhancement bias; same-model review is acceptable per Ho et al. 2025 for structured QA.</t>
         </is>
       </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>✓ NeurIPS 2023</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -625,6 +664,11 @@
           <t>LectureBench adopts G-Eval's form-filling paradigm (structured sub-scores per criterion) but grounds each score in verifiable source chunk text, limiting self-preference drift.</t>
         </is>
       </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>✓ EMNLP 2023</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -662,6 +706,11 @@
           <t>LectureBench adopts the rubric-per-criterion principle but uses Claude Sonnet 4.6 prompted with task-specific criteria rather than a fine-tuned evaluator, keeping the pipeline simple.</t>
         </is>
       </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>✓ ICLR 2024</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -699,6 +748,11 @@
           <t>Key finding directly answers Q1: same-model review is acceptable for structured QA. LectureBench can use Claude Sonnet 4.6 as both generator and reviewer without circularity risk.</t>
         </is>
       </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="40" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -736,6 +790,11 @@
           <t>Supports the general validity of LLM judges in structured evaluation pipelines; reinforces using a strong model (Claude Sonnet 4.6 or GPT-4o) as reviewer.</t>
         </is>
       </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -773,6 +832,11 @@
           <t>LectureBench reviewer verifies each answer claim against cited chunk text (analogous to FActScore's atomic verification). Frame captions convert visual content to text, enabling text-only correctness checking.</t>
         </is>
       </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>✓ EMNLP 2023</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -810,6 +874,11 @@
           <t>RAGAS's faithfulness criterion (answer claims supported by retrieved context) directly informs LectureBench's answer correctness check: the reviewer verifies each answer against cited chunk text.</t>
         </is>
       </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>✓ EACL 2024</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -847,6 +916,11 @@
           <t>Directly motivates the -10s span gap rejection criterion in LectureBench: adjacent chunks are single-hop in disguise. Reviewer must reject multi-hop questions where both spans map to the same or adjacent chunks.</t>
         </is>
       </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>✓ ACL 2019</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -884,6 +958,11 @@
           <t>Supports the LectureBench design: multi-hop questions should require separate retrieval steps from non-adjacent lecture segments, validating our adjacency rejection criterion.</t>
         </is>
       </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2024) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -921,6 +1000,11 @@
           <t>Reinforces using structured sub-criterion prompting (our form-filling approach) to mitigate SPB. Combined with Ho et al. 2025 finding of no SPB in structured QA, the LectureBench reviewer design is well-supported.</t>
         </is>
       </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="40" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -958,6 +1042,11 @@
           <t>Validates LectureBench's design choice of step-level (span-level) evaluation over answer-only metrics. Supports using span plausibility as a review criterion in Phase 7.3.</t>
         </is>
       </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -995,6 +1084,11 @@
           <t>Explains why SPB is less of a risk in LectureBench: the reviewer is verifying chunk-grounded factual claims (not stylistically similar to its training distribution), so perplexity familiarity does not apply in the same way.</t>
         </is>
       </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>✓ NeurIPS 2024 Workshop (Safe Generative AI)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="40" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -1032,6 +1126,11 @@
           <t>LectureBench's ±15–30s span precision is actually better than EduVidQA's ±35.4s. If EduVidQA is accepted without tightening, LectureBench can make the same choice and cite this precedent.</t>
         </is>
       </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>✓ EMNLP 2025</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="40" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1069,6 +1168,11 @@
           <t>Represents the ideal; LectureBench trades span precision for scale. Justifies using tIoU@0.3 as the primary threshold (more forgiving of ±15–30s error) rather than tIoU@0.5.</t>
         </is>
       </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="40" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -1106,6 +1210,11 @@
           <t>For LectureBench Phase 7.3, PCFJudge's consensus principle could be applied to C1 (answer correctness) by running the reviewer twice with shuffled claim order and requiring agreement. However, G-Eval structured form-filling already reduces order sensitivity — PCFJudge's main benefit is marginal for binary criteria.</t>
         </is>
       </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="40" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1143,6 +1252,11 @@
           <t>Confirms majority voting as the simplest and most robust aggregation strategy if multi-judge is adopted. For LectureBench, majority vote across 2 judges (Claude + GPT-4o) on borderline cases is a lightweight option if Phase 7.3 single-judge produces high disagreement rates.</t>
         </is>
       </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="40" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -1180,6 +1294,11 @@
           <t>PRD's discussion mechanism is most valuable for subjective open-ended scoring (Phase 8 LLM-judge 1-5 scale), not for Phase 7.3's binary criteria checks. For binary PASS/FAIL, simple majority vote is sufficient and cheaper.</t>
         </is>
       </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2023) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="40" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -1217,6 +1336,11 @@
           <t>ChatEval's persona diversity principle is most valuable for Phase 8 LLM-judge scoring where answer quality is subjective. For Phase 7.3's factuality checks (C1 claim verification), the task is objective enough that debate adds minimal signal over a structured single-judge prompt.</t>
         </is>
       </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>✓ ICLR 2024</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="40" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -1254,6 +1378,11 @@
           <t>Confirms the principle that multi-judge aggregation reduces bias, but the distillation approach is not practical for LectureBench. The relevant finding is that 2-3 judge majority vote achieves most of the bias reduction benefit without distillation.</t>
         </is>
       </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2025) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="40" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1291,6 +1420,11 @@
           <t>The 15-25% inconsistency finding argues for reporting judge reliability metrics (Kappa between two runs with different prompt seeds) in the paper's Phase 7.3 methodology section. This strengthens credibility without requiring a full second-model review pass.</t>
         </is>
       </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2024) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="40" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -1328,6 +1462,11 @@
           <t>For LectureBench Q4: lecture content (especially cutting-edge ML topics from MIT/Stanford/NYU) may conflict with Claude's parametric knowledge. Lee et al. (2026) argues this is a real failure mode for reference-based judging. The cross-family optional reviewer (GPT-4o) in D1 gains additional justification specifically for Q4 in lectures covering recent or specialized content. This strengthens the case for the optional Kappa reliability check (D8b): if Kappa &lt; 0.7, the disagreements are likely driven by knowledge conflicts, not random noise.</t>
         </is>
       </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>✗ arXiv preprint (2026) — not peer-reviewed</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="40" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -1365,6 +1504,11 @@
           <t>Supports Q1 decision: LLM single-judge is reliable for structured Pass/Fail tasks. Peer-reviewed alternative to the unreviewed Ho et al. (2025) preprint for structured evaluation reliability.</t>
         </is>
       </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>✓ Frontiers in Big Data (2025)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="40" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -1400,6 +1544,11 @@
       <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Supports Q2 decision: decomposed criteria-based evaluation (our G-Eval rubric with Criterion 1/2/3) achieves higher human correlation than holistic pointwise scoring. Peer-reviewed EMNLP 2025 publication strengthens rubric design justification.</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>✓ EMNLP 2025 Industry Track</t>
         </is>
       </c>
     </row>

</xml_diff>